<commit_message>
Updated code burst hackathon materials
</commit_message>
<xml_diff>
--- a/data/publicationslist_HEAL.xlsx
+++ b/data/publicationslist_HEAL.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lmaefos\Code Stuffs\spec-driven-row-wise-workflow\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19C6BD40-2A7E-4545-9432-B7B263099687}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{205188BE-C513-4B08-A65D-D340B12C2A2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15675" xr2:uid="{2151761E-8006-45FA-AF82-08BA95474834}"/>
+    <workbookView xWindow="-38505" yWindow="4500" windowWidth="19410" windowHeight="20985" xr2:uid="{2151761E-8006-45FA-AF82-08BA95474834}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="143">
   <si>
     <t>PMID</t>
   </si>
@@ -339,6 +339,138 @@
   </si>
   <si>
     <t>We sought to evaluate the impact of the coronavirus disease 2019 (COVID-19) pandemic on perinatal outcomes while accounting for maternal depression or perceived stress and to describe COVID-specific stressors, including changes in prenatal care, across specific time periods of the pandemic. Data of dyads from 41 cohorts from the National Institutes of Health Environmental influences on Child Health Outcomes Program (&lt;i&gt;N&lt;/i&gt; = 2,983) were used to compare birth outcomes before and during the pandemic (&lt;i&gt;n&lt;/i&gt; = 2,355), and a partially overlapping sample (&lt;i&gt;n&lt;/i&gt; = 1,490) responded to a COVID-19 questionnaire. Psychosocial stress was defined using prenatal screening for depression and perceived stress. Propensity-score matching and general estimating equations with robust variance estimation were used to estimate the pandemic's effect on birth outcomes. Symptoms of depression and perceived stress during pregnancy were similar prior to and during the pandemic, with nearly 40% of participants reporting mild to severe stress, and 24% reporting mild depression to severe depression. Gestations were shorter during the pandemic (&lt;i&gt;B&lt;/i&gt; =  - 0.33 weeks, &lt;i&gt;p&lt;/i&gt; = 0.025), and depression was significantly associated with shortened gestation (&lt;i&gt;B&lt;/i&gt; =  - 0.02 weeks, &lt;i&gt;p&lt;/i&gt; = 0.015) after adjustment. Birth weights were similar (&lt;i&gt;B&lt;/i&gt; =  - 28.14 g, &lt;i&gt;p&lt;/i&gt; = 0.568), but infants born during the pandemic had slightly larger birth weights for gestational age at delivery than those born before the pandemic (&lt;i&gt;B&lt;/i&gt; = 0.15 z-score units, &lt;i&gt;p&lt;/i&gt; = 0.041). More women who gave birth early in the pandemic reported being moderately or extremely distressed about changes to their prenatal care and delivery (45%) compared with those who delivered later in the pandemic. A majority (72%) reported somewhat to extremely negative views of the impact of COVID-19 on their life. In this national cohort, we detected no effect of COVID-19 on prenatal depression or perceived stress. However, experiencing the COVID-19 pandemic in pregnancy was associated with decreases in gestational age at birth, as well as distress about changes in prenatal care early in the pandemic. · COVID-19 was associated with shortened gestations.. · Depression was associated with shortened gestations.. · However, stress during the pandemic remained unchanged.. · Most women reported negative impacts of the pandemic..</t>
+  </si>
+  <si>
+    <t>37515516</t>
+  </si>
+  <si>
+    <t>PMC10823040</t>
+  </si>
+  <si>
+    <t>10.1002/jmri.28907</t>
+  </si>
+  <si>
+    <t>Motion Robust MR Fingerprinting Scan to Image Neonates With Prenatal Opioid Exposure.</t>
+  </si>
+  <si>
+    <t>To explore whether MR fingerprinting (MRF) scans provide motion-robust and quantitative brain tissue measurements for non-sedated infants with prenatal opioid exposure (POE). Prospective. 13 infants with POE (3 male; 12 newborns (age 7-65 days) and 1 infant aged 9-months). 3T, 3D T1-weighted MPRAGE, 3D T2-weighted TSE and MRF sequences. The image quality of MRF and MRI was assessed in a fully crossed, multiple-reader, multiple-case study. Sixteen image quality features in three types-image artifacts, structure and myelination visualization-were ranked by four neuroradiologists (8, 7, 5, and 8 years of experience respectively), using a 3-point scale. MRF T1 and T2 values in 8 white matter brain regions were compared between babies younger than 1 month and babies between 1 and 2 months. Generalized estimating equations model to test the significance of differences of regional T1 and T2 values of babies under 1 month and those older. MRI and MRF image quality was assessed using Gwet's second order auto-correlation coefficient (AC&lt;sub&gt;2&lt;/sub&gt;) with confidence levels. The Cochran-Mantel-Haenszel test was used to assess the difference in proportions between MRF and MRI for all features and stratified by the type of features. A P value &lt;0.05 was considered statistically significant. The MRF of two infants were excluded in T1 and T2 value analysis due to severe motion artifact but were included in the image quality assessment. In infants under 1 month of age (N = 6), the T1 and T2 values were significantly higher compared to those between 1 and 2 months of age (N = 4). MRF images showed significantly higher image quality ratings in all three feature types compared to MRI images. MR Fingerprinting scans have potential to be a motion-robust and efficient method for nonsedated infants. 2 TECHNICAL EFFICACY STAGE: 1.</t>
+  </si>
+  <si>
+    <t>37963235</t>
+  </si>
+  <si>
+    <t>PMC10950549</t>
+  </si>
+  <si>
+    <t>10.1097/j.pain.0000000000003090</t>
+  </si>
+  <si>
+    <t>A phenotypic screening platform for chronic pain therapeutics using all-optical electrophysiology.</t>
+  </si>
+  <si>
+    <t>Chronic pain associated with osteoarthritis (OA) remains an intractable problem with few effective treatment options. New approaches are needed to model the disease biology and to drive discovery of therapeutics. We present an in vitro model of OA pain, where dorsal root ganglion (DRG) sensory neurons were sensitized by a defined mixture of disease-relevant inflammatory mediators, here called Sensitizing PAin Reagent Composition or SPARC. Osteoarthritis-SPARC components showed synergistic or additive effects when applied in combination and induced pain phenotypes in vivo. To measure the effect of OA-SPARC on neural firing in a scalable format, we used a custom system for high throughput all-optical electrophysiology. This system enabled light-based membrane voltage recordings from hundreds of neurons in parallel with single cell and single action potential resolution and a throughput of up to 500,000 neurons per day. A computational framework was developed to construct a multiparameter OA-SPARC neuronal phenotype and to quantitatively assess phenotype reversal by candidate pharmacology. We screened ∼3000 approved drugs and mechanistically focused compounds, yielding data from over 1.2 million individual neurons with detailed assessment of functional OA-SPARC phenotype rescue and orthogonal "off-target" effects. Analysis of confirmed hits revealed diverse potential analgesic mechanisms including ion channel modulators and other mechanisms including MEK inhibitors and tyrosine kinase modulators. Our results suggest that the Raf-MEK-ERK axis in DRG neurons may integrate the inputs from multiple upstream inflammatory mediators found in osteoarthritis patient joints, and MAPK pathway activation in DRG neurons may contribute to chronic pain in patients with osteoarthritis.</t>
+  </si>
+  <si>
+    <t>37731248</t>
+  </si>
+  <si>
+    <t>PMC10950840</t>
+  </si>
+  <si>
+    <t>10.1111/jsr.14037</t>
+  </si>
+  <si>
+    <t>Biological sex influences sleep phenotype in mice experiencing spontaneous opioid withdrawal.</t>
+  </si>
+  <si>
+    <t>Aversive symptoms, including insomnia experienced during opioid withdrawal, are a major drive to relapse; however, withdrawal-associated sleep symptomatology has been little explored in preclinical models. We describe here a model of opioid withdrawal in mice that resembles the sleep phenotype characteristic of withdrawal in humans. Male and female C57BL/6 mice were instrumented with telemeters to record electroencephalogram, electromyogram, activity and subcutaneous temperature. All mice received two treatments separated by a 16-day washout period: (1) saline (volume: 10 ml kg&lt;sup&gt;-1&lt;/sup&gt;); or (2) ascending doses of morphine (5, 10, 20, 40 and 80 mg kg&lt;sup&gt;-1&lt;/sup&gt;; volume: 10 ml kg&lt;sup&gt;-1&lt;/sup&gt;) for 5 days at Zeitgeber time 1 and Zeitgeber time 13. Recordings for the first 71 hr after treatment discontinuation (withdrawal days 1-3) and for 24 hr on withdrawal days 5 and 7 were scored for sleep/wake state, and sleep architecture and electroencephalogram spectral data were analysed. Morphine was acutely wake- and activity-promoting, and non-rapid eye movement and rapid eye movement sleep were increased during the dark phase on withdrawal day 2 in both sexes. While non-rapid eye movement delta power (0.5-4.0 Hz), a measure of sleep intensity, was reduced during the light phase on withdrawal day 1 and the dark phase on withdrawal day 2 in both sexes, female mice also exhibited changes in the duration and the number of bouts of sleep/wake states. These observations of fragmented sleep on withdrawal days 1-3 suggest poorer sleep consolidation and a more pronounced withdrawal-associated sleep phenotype in female than in male mice. These data may indicate a greater sensitivity to morphine, a more distinct aversive sleep phenotype and/or a faster escalation to dependence in female mice.</t>
+  </si>
+  <si>
+    <t>38109146</t>
+  </si>
+  <si>
+    <t>PMC10984762</t>
+  </si>
+  <si>
+    <t>10.1002/jts.23000</t>
+  </si>
+  <si>
+    <t>Longitudinal associations among experiences of sexual assault, posttraumatic stress disorder symptoms, and heavy drinking in young adults.</t>
+  </si>
+  <si>
+    <t>Prior research with young adults has demonstrated clear associations between experiences of sexual assault, symptoms of posttraumatic stress disorder (PTSD), and alcohol use, but most studies have been cross-sectional or have not considered multiple theoretical pathways to understand these associations. Using six waves of data from a longitudinal cohort sample of 1,719 young adults, we examined associations among experiences of past-year sexual assault (i.e., rape, unwanted sexual touching, and physical intimidation in a sexual way), PTSD symptoms, and the frequency of binge drinking over time, allowing for the exploration of symptom-induced, interpersonal risk, and substance-induced pathways for male and female participants. For both male, βs = 2.84 to 6.55, and female participants, βs = 2.96 to 10.1, higher prior levels of PTSD symptoms were associated with larger increases in binge drinking over time. For female participants, higher prior levels of sexual assault were associated with larger increases in PTSD symptoms over time, βs = 3.48 to 4.25, whereas for male participants, higher prior levels of past-year binge drinking were associated with decreases in PTSD symptoms over time, βs = -2.75 to -0.53. Continued efforts are needed to prevent sexual assault among young adults and address PTSD symptoms among those who experience sexual assault. Interventions that target binge drinking are also needed for individuals who experience PTSD symptoms, especially young adults, to address potentially hazardous drinking before problems escalate and become chronic.</t>
+  </si>
+  <si>
+    <t>37923885</t>
+  </si>
+  <si>
+    <t>PMC10891245</t>
+  </si>
+  <si>
+    <t>10.1007/s11121-023-01612-3</t>
+  </si>
+  <si>
+    <t>Mixed Methods Evaluation of Satisfaction with Two Culturally Tailored Substance use Prevention Programs for American Indian/Alaska Native Emerging Adults.</t>
+  </si>
+  <si>
+    <t>American Indian/Alaska Native (AI/AN) communities are disproportionately affected by the opioid epidemic. AI/AN emerging adults (ages 18-25) in urban areas are at particularly high risk, with the overdose death rate among urban-dwelling AI/AN people 1.4 times higher than rural-dwelling AI/AN people. Despite these challenges, there are no evidence-based culturally tailored prevention or intervention programs to address opioid, alcohol and other drug use among urban AI/AN emerging adults. This study focused on understanding AI/AN emerging adults' experiences with two culturally tailored programs addressing opioid, cannabis, and alcohol use as part of the randomized controlled trial for Traditions and Connections for Urban Native Americans (TACUNA) in order to enhance feasibility of this intervention. Using a convergent mixed methods design at 3-month follow-up, we collected satisfaction and experience ratings and written narratives (total n = 162; intervention n = 77; control n = 85) from a sample of urban-dwelling AI/AN emerging adults who participated in both programs. We analyzed data through simultaneous examination of qualitative and quantitative data. The quantitative ratings show that both programs were rated highly. The qualitative data contextualized these ratings, illustrating pathways through which specific components were perceived to cause desired or observed behavioral change in participants. Among the elements that mattered most to these participants were the convenience of the virtual format, having a comfortable and safe space to share personal stories, and learning new information about their social networks. Negative comments focused on workshop length and inconvenient scheduling. This is one of the first studies to explore participant satisfaction and experience with culturally tailored substance use programming among a historically marginalized and understudied population. It is important to consider the voices of urban-dwelling AI/AN people in program development because hidden factors, such as limited financial resources, limited time, and misalignment with cultural values may prevent existing programs from being feasible.</t>
+  </si>
+  <si>
+    <t>37877647</t>
+  </si>
+  <si>
+    <t>10.1111/papr.13309</t>
+  </si>
+  <si>
+    <t>Pandemic impact and adaptation to telehealth in chronic pain treatment providers across two COVID-19 pandemic years.</t>
+  </si>
+  <si>
+    <t>The COVID-19 pandemic has had substantial impacts for both people using pain services and healthcare professionals delivering them. While the effects on service users have been studied, less is known about the effects for service providers. This study aimed to assess the impact of the pandemic on providers and the evolving role of telemedicine in treatment. An electronic survey was distributed to the professional membership of the European Pain Federation (EFIC). The survey evaluated impact and adjustment to the COVID-19 pandemic separately across two pandemic years (March 2020-February 2021 and March 2021 to February 2022) and assessed worry about COVID-19, disruption and adjustment of pain services, and use of telehealth services. The change between the first and second pandemic years and the degree to which telehealth services were adopted was evaluated. From 149 respondents, 131 (88%) participants provided sufficient data to be included in the analysis. Both providers worry about the pandemic and service disruption decreased significantly from the first to the second year of the pandemic. Prior to the pandemic, only 30% of providers offered telehealth appointments but this increased to 64% and 83%, respectively, in the first and second years of the pandemic. Although provider worry and disruption to delivery of pain services decreased during the second year of COVID-19 pandemic, waiting times for appointments continued to lengthen. The pandemic has hastened the adoption of telemedicine in pain services and plans to continue telehealth services seem common.</t>
+  </si>
+  <si>
+    <t>38011858</t>
+  </si>
+  <si>
+    <t>PMC11162597</t>
+  </si>
+  <si>
+    <t>10.1111/add.16394</t>
+  </si>
+  <si>
+    <t>Performance of International Classification of Disease-10 codes in detecting emergency department patients with opioid misuse.</t>
+  </si>
+  <si>
+    <t>Accurate case discovery is critical for disease surveillance, resource allocation and research. International Classification of Disease (ICD) diagnosis codes are commonly used for this purpose. We aimed to determine the sensitivity, specificity and positive predictive value (PPV) of ICD-10 codes for opioid misuse case discovery in the emergency department (ED) setting. Retrospective cohort study of ED encounters from January 2018 to December 2020 at an urban academic hospital in the United States. A sample of ED encounters enriched for opioid misuse was developed by oversampling ED encounters with positive urine opiate screens or pre-existing opioid-related diagnosis codes in addition to other opioid misuse risk factors. A total of 1200 randomly selected encounters were annotated by research staff for the presence of opioid misuse within health record documentation using a 5-point scale for likelihood of opioid misuse and dichotomized into cohorts of opioid misuse and no opioid misuse. Using manual annotation as ground truth, the sensitivity and specificity of ICD-10 codes entered during the encounter were determined with PPV adjusted for oversampled data. Metrics were also determined by disposition subgroup: discharged home or admitted. There were 541 encounters annotated as opioid misuse and 617 with no opioid misuse. The majority were males (54.4%), average age was 47 years and 68.5% were discharged directly from the ED. The sensitivity of ICD-10 codes was 0.56 (95% confidence interval [CI], 0.51-0.60), specificity 0.99 (95% CI, 0.97-0.99) and adjusted PPV 0.78 (95% CI, 0.65-0.92). The sensitivity was higher for patients discharged from the ED (0.65; 95% CI, 0.60-0.69) than those admitted (0.31; 95% CI, 0.24-0.39). International Classification of Disease-10 codes appear to have low sensitivity but high specificity and positive predictive value in detecting opioid misuse among emergency department patients in the United States.</t>
+  </si>
+  <si>
+    <t>37955711</t>
+  </si>
+  <si>
+    <t>PMC10933137</t>
+  </si>
+  <si>
+    <t>10.1007/s00737-023-01390-5</t>
+  </si>
+  <si>
+    <t>Psychological distress among postpartum women who took opioids during pregnancy: the role of perceived stigma in healthcare settings.</t>
+  </si>
+  <si>
+    <t>This study examined the relationship between perceived stigma in healthcare settings during pregnancy and psychological distress and well-being in the postpartum period among individuals who took opioids while pregnant. Analyses included 134 birth mothers of opioid-exposed infants. At 0-1 months postpartum, perceived stigma and psychological distress were measured using the Prenatal Opioid use Perceived Stigma scale and measures from the Patient-Reported Outcome Measurement Information System (PROMIS). Food insecurity, housing instability, and Adverse Childhood Experiences (ACEs) were also assessed. Linear and generalized linear mixed-effect models were conducted to compare PROMIS scale scores and unmet needs by stigma, adjusting for site/location, age, race/ethnicity, marital status, education, public insurance, and parity. More than half of participants (54%) perceived stigma in healthcare settings. Individuals reporting stigma had higher depression, anxiety, and anger scores (p &lt; 0.001) indicating greater psychological distress in the postpartum period compared to those reporting no stigma, after controlling for demographic characteristics. In addition, they scored significantly lower on the PROMIS meaning and purpose scale, an indicator of well-being (p = 0.002). Those reporting stigma were more likely to have food insecurity (p = 0.003), three or more ACEs (p = 0.040), verbal or physical abuse during pregnancy (p &lt; 0.001), and less emotional support (p = 0.006) than those who did not. An association was observed between perceived stigma in the prenatal period and psychological distress in the postpartum period, providing support for stigma reduction interventions and education for healthcare providers on trauma-informed care.</t>
+  </si>
+  <si>
+    <t>37675827</t>
+  </si>
+  <si>
+    <t>PMC10921423</t>
+  </si>
+  <si>
+    <t>10.1002/adbi.202300276</t>
+  </si>
+  <si>
+    <t>Human IPSC-Derived PreBötC-Like Neurons and Development of an Opiate Overdose and Recovery Model.</t>
+  </si>
+  <si>
+    <t>Opioid overdose is the leading cause of drug overdose lethality, posing an urgent need for investigation. The key brain region for inspiratory rhythm regulation and opioid-induced respiratory depression (OIRD) is the preBötzinger Complex (preBötC) and current knowledge has mainly been obtained from animal systems. This study aims to establish a protocol to generate human preBötC neurons from induced pluripotent cells (iPSCs) and develop an opioid overdose and recovery model utilizing these iPSC-preBötC neurons. A de novo protocol to differentiate preBötC-like neurons from human iPSCs is established. These neurons express essential preBötC markers analyzed by immunocytochemistry and demonstrate expected electrophysiological responses to preBötC modulators analyzed by patch clamp electrophysiology. The correlation of the specific biomarkers and function analysis strongly suggests a preBötC-like phenotype. Moreover, the dose-dependent inhibition of these neurons' activity is demonstrated for four different opioids with identified IC50's comparable to the literature. Inhibition is rescued by naloxone in a concentration-dependent manner. This iPSC-preBötC mimic is crucial for investigating OIRD and combating the overdose crisis and a first step for the integration of a functional overdose model into microphysiological systems.</t>
   </si>
 </sst>
 </file>
@@ -406,7 +538,18 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="1">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -736,7 +879,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ADBA81DC-F5BA-4F52-8E1A-46E5FC9DF721}">
-  <dimension ref="A1:E20"/>
+  <dimension ref="A1:E29"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="9.796875" bestFit="1" customWidth="1"/>
@@ -1086,8 +1229,164 @@
         <v>98</v>
       </c>
     </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A21" t="s">
+        <v>99</v>
+      </c>
+      <c r="B21" t="s">
+        <v>100</v>
+      </c>
+      <c r="C21" t="s">
+        <v>101</v>
+      </c>
+      <c r="D21" t="s">
+        <v>102</v>
+      </c>
+      <c r="E21" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A22" t="s">
+        <v>104</v>
+      </c>
+      <c r="B22" t="s">
+        <v>105</v>
+      </c>
+      <c r="C22" t="s">
+        <v>106</v>
+      </c>
+      <c r="D22" t="s">
+        <v>107</v>
+      </c>
+      <c r="E22" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A23" t="s">
+        <v>109</v>
+      </c>
+      <c r="B23" t="s">
+        <v>110</v>
+      </c>
+      <c r="C23" t="s">
+        <v>111</v>
+      </c>
+      <c r="D23" t="s">
+        <v>112</v>
+      </c>
+      <c r="E23" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A24" t="s">
+        <v>114</v>
+      </c>
+      <c r="B24" t="s">
+        <v>115</v>
+      </c>
+      <c r="C24" t="s">
+        <v>116</v>
+      </c>
+      <c r="D24" t="s">
+        <v>117</v>
+      </c>
+      <c r="E24" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A25" t="s">
+        <v>119</v>
+      </c>
+      <c r="B25" t="s">
+        <v>120</v>
+      </c>
+      <c r="C25" t="s">
+        <v>121</v>
+      </c>
+      <c r="D25" t="s">
+        <v>122</v>
+      </c>
+      <c r="E25" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A26" t="s">
+        <v>124</v>
+      </c>
+      <c r="B26" t="s">
+        <v>31</v>
+      </c>
+      <c r="C26" t="s">
+        <v>125</v>
+      </c>
+      <c r="D26" t="s">
+        <v>126</v>
+      </c>
+      <c r="E26" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A27" t="s">
+        <v>128</v>
+      </c>
+      <c r="B27" t="s">
+        <v>129</v>
+      </c>
+      <c r="C27" t="s">
+        <v>130</v>
+      </c>
+      <c r="D27" t="s">
+        <v>131</v>
+      </c>
+      <c r="E27" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A28" t="s">
+        <v>133</v>
+      </c>
+      <c r="B28" t="s">
+        <v>134</v>
+      </c>
+      <c r="C28" t="s">
+        <v>135</v>
+      </c>
+      <c r="D28" t="s">
+        <v>136</v>
+      </c>
+      <c r="E28" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A29" t="s">
+        <v>138</v>
+      </c>
+      <c r="B29" t="s">
+        <v>139</v>
+      </c>
+      <c r="C29" t="s">
+        <v>140</v>
+      </c>
+      <c r="D29" t="s">
+        <v>141</v>
+      </c>
+      <c r="E29" t="s">
+        <v>142</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:E20" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <conditionalFormatting sqref="A1:A1048576">
+    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>